<commit_message>
Adds better .xlsx formatting. Adds auto detection for maximum current. Adds faster and more precise torque limits.
</commit_message>
<xml_diff>
--- a/Alwin-RMTest-T107357.xlsx
+++ b/Alwin-RMTest-T107357.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -32,24 +32,6 @@
   </si>
   <si>
     <t>Linearität</t>
-  </si>
-  <si>
-    <t>Mittelposition</t>
-  </si>
-  <si>
-    <t>Start aktiver Bereich CW (Drehrichtung-)</t>
-  </si>
-  <si>
-    <t>50° CW (25% aktiver Bereich)(Drehrichtung-)</t>
-  </si>
-  <si>
-    <t>75° CW (50% aktiver Bereich)(Drehrichtung-)</t>
-  </si>
-  <si>
-    <t>100° CW (75% aktiver Bereich)(Drehrichtung-)</t>
-  </si>
-  <si>
-    <t>Ende aktiver Bereich CW (Drehrichtung-)(11) 10V</t>
   </si>
   <si>
     <t>Mechanisches Ende CW (Drehrichtung-)</t>
@@ -77,10 +59,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0,0°"/>
-    <numFmt numFmtId="165" formatCode="0,000"/>
-    <numFmt numFmtId="166" formatCode="0,00%"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.0°"/>
+    <numFmt numFmtId="165" formatCode="0.00"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -134,11 +117,20 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -436,33 +428,34 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F14"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
     <col min="2" max="2" width="20.7109375" style="1" customWidth="1"/>
-    <col min="3" max="4" width="20.7109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="20.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="3" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" style="1" customWidth="1"/>
-    <col min="6" max="6" width="20.7109375" style="3" customWidth="1"/>
+    <col min="6" max="6" width="20.7109375" style="4" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
     </row>
@@ -476,13 +469,13 @@
       <c r="C2" s="2">
         <v>5</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="3">
         <v>3</v>
       </c>
       <c r="E2" s="1">
-        <v>-0</v>
-      </c>
-      <c r="F2" s="3">
+        <v>-0.1</v>
+      </c>
+      <c r="F2" s="4">
         <v>-0.2</v>
       </c>
     </row>
@@ -496,13 +489,13 @@
       <c r="C3" s="2">
         <v>5</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="3">
         <v>4</v>
       </c>
       <c r="E3" s="1">
-        <v>24.4</v>
-      </c>
-      <c r="F3" s="3">
+        <v>24.3</v>
+      </c>
+      <c r="F3" s="4">
         <v>-0.1</v>
       </c>
     </row>
@@ -516,13 +509,13 @@
       <c r="C4" s="2">
         <v>6.25</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="3">
         <v>4</v>
       </c>
       <c r="E4" s="1">
-        <v>49.4</v>
-      </c>
-      <c r="F4" s="3">
+        <v>49.3</v>
+      </c>
+      <c r="F4" s="4">
         <v>-0.22</v>
       </c>
     </row>
@@ -536,13 +529,13 @@
       <c r="C5" s="2">
         <v>7.5</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="3">
         <v>5</v>
       </c>
       <c r="E5" s="1">
-        <v>74.40000000000001</v>
-      </c>
-      <c r="F5" s="3">
+        <v>74.3</v>
+      </c>
+      <c r="F5" s="4">
         <v>-0.25</v>
       </c>
     </row>
@@ -556,13 +549,13 @@
       <c r="C6" s="2">
         <v>8.75</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="3">
         <v>6</v>
       </c>
       <c r="E6" s="1">
         <v>99.3</v>
       </c>
-      <c r="F6" s="3">
+      <c r="F6" s="4">
         <v>-0.27</v>
       </c>
     </row>
@@ -576,13 +569,13 @@
       <c r="C7" s="2">
         <v>10</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="3">
         <v>6</v>
       </c>
       <c r="E7" s="1">
-        <v>124.4</v>
-      </c>
-      <c r="F7" s="3">
+        <v>124.3</v>
+      </c>
+      <c r="F7" s="4">
         <v>-0.4</v>
       </c>
     </row>
@@ -596,134 +589,14 @@
       <c r="C8" s="2">
         <v>10</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="3">
         <v>7</v>
       </c>
       <c r="E8" s="1">
         <v>165.5</v>
       </c>
-      <c r="F8" s="3">
+      <c r="F8" s="4">
         <v>-0.3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" s="1">
-        <v>-25</v>
-      </c>
-      <c r="C9" s="2">
-        <v>5</v>
-      </c>
-      <c r="D9" s="2">
-        <v>3</v>
-      </c>
-      <c r="E9" s="1">
-        <v>-25.6</v>
-      </c>
-      <c r="F9" s="3">
-        <v>-0.2</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" s="1">
-        <v>-50</v>
-      </c>
-      <c r="C10" s="2">
-        <v>3.75</v>
-      </c>
-      <c r="D10" s="2">
-        <v>2</v>
-      </c>
-      <c r="E10" s="1">
-        <v>-50.7</v>
-      </c>
-      <c r="F10" s="3">
-        <v>-0.17</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" s="1">
-        <v>-75</v>
-      </c>
-      <c r="C11" s="2">
-        <v>2.5</v>
-      </c>
-      <c r="D11" s="2">
-        <v>2</v>
-      </c>
-      <c r="E11" s="1">
-        <v>-75.59999999999999</v>
-      </c>
-      <c r="F11" s="3">
-        <v>-0.05</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" t="s">
-        <v>16</v>
-      </c>
-      <c r="B12" s="1">
-        <v>-100</v>
-      </c>
-      <c r="C12" s="2">
-        <v>1.25</v>
-      </c>
-      <c r="D12" s="2">
-        <v>1</v>
-      </c>
-      <c r="E12" s="1">
-        <v>-100.6</v>
-      </c>
-      <c r="F12" s="3">
-        <v>-0.03</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" t="s">
-        <v>17</v>
-      </c>
-      <c r="B13" s="1">
-        <v>-125</v>
-      </c>
-      <c r="C13" s="2">
-        <v>0</v>
-      </c>
-      <c r="D13" s="2">
-        <v>0</v>
-      </c>
-      <c r="E13" s="1">
-        <v>-125.7</v>
-      </c>
-      <c r="F13" s="3">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" t="s">
-        <v>18</v>
-      </c>
-      <c r="B14" s="1">
-        <v>-165.6</v>
-      </c>
-      <c r="C14" s="2">
-        <v>0</v>
-      </c>
-      <c r="D14" s="2">
-        <v>0</v>
-      </c>
-      <c r="E14" s="1">
-        <v>-165.6</v>
-      </c>
-      <c r="F14" s="3">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds Smoother state switching between current measuring and position measuring. Calculates internally in ticks instead of degrees. User Input and Output still in degrees for ease of reading. Adds instant cancel at any point during automatic measurement.
</commit_message>
<xml_diff>
--- a/Alwin-RMTest-T107357.xlsx
+++ b/Alwin-RMTest-T107357.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t xml:space="preserve"> </t>
   </si>
@@ -32,6 +32,24 @@
   </si>
   <si>
     <t>Linearität</t>
+  </si>
+  <si>
+    <t>Mittelposition</t>
+  </si>
+  <si>
+    <t>Start aktiver Bereich CW (Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>50° CW (25% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>75° CW (50% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>100° CW (75% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>Ende aktiver Bereich CW (Drehrichtung-)(11) 10V</t>
   </si>
   <si>
     <t>Mechanisches Ende CW (Drehrichtung-)</t>
@@ -428,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -470,13 +488,13 @@
         <v>5</v>
       </c>
       <c r="D2" s="3">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E2" s="1">
-        <v>-0.1</v>
+        <v>-0</v>
       </c>
       <c r="F2" s="4">
-        <v>-0.2</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -490,13 +508,13 @@
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E3" s="1">
-        <v>24.3</v>
+        <v>24.9</v>
       </c>
       <c r="F3" s="4">
-        <v>-0.1</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -510,13 +528,13 @@
         <v>6.25</v>
       </c>
       <c r="D4" s="3">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E4" s="1">
-        <v>49.3</v>
+        <v>50</v>
       </c>
       <c r="F4" s="4">
-        <v>-0.22</v>
+        <v>-0.32</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -530,13 +548,13 @@
         <v>7.5</v>
       </c>
       <c r="D5" s="3">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E5" s="1">
-        <v>74.3</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="F5" s="4">
-        <v>-0.25</v>
+        <v>-0.45</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -550,13 +568,13 @@
         <v>8.75</v>
       </c>
       <c r="D6" s="3">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E6" s="1">
-        <v>99.3</v>
+        <v>99.90000000000001</v>
       </c>
       <c r="F6" s="4">
-        <v>-0.27</v>
+        <v>-0.47</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -570,13 +588,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="3">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E7" s="1">
-        <v>124.3</v>
+        <v>125</v>
       </c>
       <c r="F7" s="4">
-        <v>-0.4</v>
+        <v>-0.5</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -590,13 +608,133 @@
         <v>10</v>
       </c>
       <c r="D8" s="3">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="1">
-        <v>165.5</v>
+        <v>165.6</v>
       </c>
       <c r="F8" s="4">
-        <v>-0.3</v>
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1">
+        <v>-25</v>
+      </c>
+      <c r="C9" s="2">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-25</v>
+      </c>
+      <c r="F9" s="4">
+        <v>-0.4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1">
+        <v>-50</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>1</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-50</v>
+      </c>
+      <c r="F10" s="4">
+        <v>-0.28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-75</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="3">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1">
+        <v>-74.90000000000001</v>
+      </c>
+      <c r="F11" s="4">
+        <v>-0.25</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="1">
+        <v>-100</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="1">
+        <v>-99.90000000000001</v>
+      </c>
+      <c r="F12" s="4">
+        <v>-0.13</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="1">
+        <v>-125</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>-125</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="1">
+        <v>-165.6</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>-1</v>
+      </c>
+      <c r="E14" s="1">
+        <v>-165.6</v>
+      </c>
+      <c r="F14" s="4">
+        <v>-0.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Adds better structuring and logo insert in Python GUI. Adds mechanical translation between pot and servo. Adds local preset .json for ease of data inserts. Adds dropdown for user friendliness.
</commit_message>
<xml_diff>
--- a/Alwin-RMTest-T107357.xlsx
+++ b/Alwin-RMTest-T107357.xlsx
@@ -488,13 +488,13 @@
         <v>5</v>
       </c>
       <c r="D2" s="3">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E2" s="1">
         <v>-0</v>
       </c>
       <c r="F2" s="4">
-        <v>-0.3</v>
+        <v>-0.1</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -508,13 +508,13 @@
         <v>5</v>
       </c>
       <c r="D3" s="3">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E3" s="1">
-        <v>24.9</v>
+        <v>25</v>
       </c>
       <c r="F3" s="4">
-        <v>-0.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -528,13 +528,13 @@
         <v>6.25</v>
       </c>
       <c r="D4" s="3">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E4" s="1">
-        <v>50</v>
+        <v>49.9</v>
       </c>
       <c r="F4" s="4">
-        <v>-0.32</v>
+        <v>-0.13</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -548,13 +548,13 @@
         <v>7.5</v>
       </c>
       <c r="D5" s="3">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E5" s="1">
         <v>74.90000000000001</v>
       </c>
       <c r="F5" s="4">
-        <v>-0.45</v>
+        <v>-0.15</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -568,13 +568,13 @@
         <v>8.75</v>
       </c>
       <c r="D6" s="3">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E6" s="1">
         <v>99.90000000000001</v>
       </c>
       <c r="F6" s="4">
-        <v>-0.47</v>
+        <v>-0.28</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -588,13 +588,13 @@
         <v>10</v>
       </c>
       <c r="D7" s="3">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E7" s="1">
         <v>125</v>
       </c>
       <c r="F7" s="4">
-        <v>-0.5</v>
+        <v>-0.3</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -608,13 +608,13 @@
         <v>10</v>
       </c>
       <c r="D8" s="3">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E8" s="1">
-        <v>165.6</v>
+        <v>165.5</v>
       </c>
       <c r="F8" s="4">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -628,13 +628,13 @@
         <v>5</v>
       </c>
       <c r="D9" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E9" s="1">
         <v>-25</v>
       </c>
       <c r="F9" s="4">
-        <v>-0.4</v>
+        <v>-0.2</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -648,13 +648,13 @@
         <v>3.75</v>
       </c>
       <c r="D10" s="3">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E10" s="1">
         <v>-50</v>
       </c>
       <c r="F10" s="4">
-        <v>-0.28</v>
+        <v>-0.08</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -668,13 +668,13 @@
         <v>2.5</v>
       </c>
       <c r="D11" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E11" s="1">
         <v>-74.90000000000001</v>
       </c>
       <c r="F11" s="4">
-        <v>-0.25</v>
+        <v>-0.05</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -688,13 +688,13 @@
         <v>1.25</v>
       </c>
       <c r="D12" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E12" s="1">
         <v>-99.90000000000001</v>
       </c>
       <c r="F12" s="4">
-        <v>-0.13</v>
+        <v>0.08</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -708,13 +708,13 @@
         <v>0</v>
       </c>
       <c r="D13" s="3">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" s="1">
         <v>-125</v>
       </c>
       <c r="F13" s="4">
-        <v>0</v>
+        <v>0.1</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -728,13 +728,13 @@
         <v>0</v>
       </c>
       <c r="D14" s="3">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="E14" s="1">
         <v>-165.6</v>
       </c>
       <c r="F14" s="4">
-        <v>-0.1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Code optimization. Adds slow/med/fast speeds for measuring.
</commit_message>
<xml_diff>
--- a/Alwin-RMTest-T107357.xlsx
+++ b/Alwin-RMTest-T107357.xlsx
@@ -13,6 +13,68 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+  <si>
+    <t xml:space="preserve"> </t>
+  </si>
+  <si>
+    <t>Soll-Winkel [°]</t>
+  </si>
+  <si>
+    <t>Soll-Spannung [V]</t>
+  </si>
+  <si>
+    <t>Ist-Spannung [V]</t>
+  </si>
+  <si>
+    <t>Ist-Winkel [°]</t>
+  </si>
+  <si>
+    <t>Linearität</t>
+  </si>
+  <si>
+    <t>Mittelposition</t>
+  </si>
+  <si>
+    <t>Start aktiver Bereich CW (Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>50° CW (25% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>75° CW (50% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>100° CW (75% aktiver Bereich)(Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>Ende aktiver Bereich CW (Drehrichtung-)(11) 10V</t>
+  </si>
+  <si>
+    <t>Mechanisches Ende CW (Drehrichtung-)</t>
+  </si>
+  <si>
+    <t>Start aktiver Bereich CCW (Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>50° CCW (25% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>75° CCW (50% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>100° CCW (75% aktiver Bereich)(Drehrichtung+)</t>
+  </si>
+  <si>
+    <t>Ende aktiver Bereich CCW (Drehrichtung+)(13) 0V</t>
+  </si>
+  <si>
+    <t>Mechanisches Ende CCW (Drehrichtung+)</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="4">
@@ -21,8 +83,16 @@
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00%"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -38,7 +108,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -46,11 +116,26 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -63,6 +148,9 @@
     </xf>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -358,7 +446,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="B1:F1"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="44.7109375" customWidth="1"/>
@@ -368,7 +456,288 @@
     <col min="5" max="5" width="20.7109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="20.7109375" style="4" customWidth="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="5" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="5" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="5" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2">
+        <v>5</v>
+      </c>
+      <c r="D2" s="3">
+        <v>5.07</v>
+      </c>
+      <c r="E2" s="1">
+        <v>0</v>
+      </c>
+      <c r="F2" s="4">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="1">
+        <v>25</v>
+      </c>
+      <c r="C3" s="2">
+        <v>5</v>
+      </c>
+      <c r="D3" s="3">
+        <v>5.07</v>
+      </c>
+      <c r="E3" s="1">
+        <v>25.1</v>
+      </c>
+      <c r="F3" s="4">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="1">
+        <v>50</v>
+      </c>
+      <c r="C4" s="2">
+        <v>6.25</v>
+      </c>
+      <c r="D4" s="3">
+        <v>6.27</v>
+      </c>
+      <c r="E4" s="1">
+        <v>50</v>
+      </c>
+      <c r="F4" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B5" s="1">
+        <v>75</v>
+      </c>
+      <c r="C5" s="2">
+        <v>7.5</v>
+      </c>
+      <c r="D5" s="3">
+        <v>7.51</v>
+      </c>
+      <c r="E5" s="1">
+        <v>75.09999999999999</v>
+      </c>
+      <c r="F5" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="1">
+        <v>100</v>
+      </c>
+      <c r="C6" s="2">
+        <v>8.75</v>
+      </c>
+      <c r="D6" s="3">
+        <v>8.76</v>
+      </c>
+      <c r="E6" s="1">
+        <v>100.1</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="1">
+        <v>125</v>
+      </c>
+      <c r="C7" s="2">
+        <v>10</v>
+      </c>
+      <c r="D7" s="3">
+        <v>10</v>
+      </c>
+      <c r="E7" s="1">
+        <v>125</v>
+      </c>
+      <c r="F7" s="4">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" t="s">
+        <v>12</v>
+      </c>
+      <c r="B8" s="1">
+        <v>166</v>
+      </c>
+      <c r="C8" s="2">
+        <v>10</v>
+      </c>
+      <c r="D8" s="3">
+        <v>10</v>
+      </c>
+      <c r="E8" s="1">
+        <v>166</v>
+      </c>
+      <c r="F8" s="4">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" s="1">
+        <v>-25</v>
+      </c>
+      <c r="C9" s="2">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>4.88</v>
+      </c>
+      <c r="E9" s="1">
+        <v>-25</v>
+      </c>
+      <c r="F9" s="4">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" t="s">
+        <v>14</v>
+      </c>
+      <c r="B10" s="1">
+        <v>-50</v>
+      </c>
+      <c r="C10" s="2">
+        <v>3.75</v>
+      </c>
+      <c r="D10" s="3">
+        <v>3.66</v>
+      </c>
+      <c r="E10" s="1">
+        <v>-50</v>
+      </c>
+      <c r="F10" s="4">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" t="s">
+        <v>15</v>
+      </c>
+      <c r="B11" s="1">
+        <v>-75</v>
+      </c>
+      <c r="C11" s="2">
+        <v>2.5</v>
+      </c>
+      <c r="D11" s="3">
+        <v>2.44</v>
+      </c>
+      <c r="E11" s="1">
+        <v>-74.90000000000001</v>
+      </c>
+      <c r="F11" s="4">
+        <v>-0.01</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" t="s">
+        <v>16</v>
+      </c>
+      <c r="B12" s="1">
+        <v>-100</v>
+      </c>
+      <c r="C12" s="2">
+        <v>1.25</v>
+      </c>
+      <c r="D12" s="3">
+        <v>1.21</v>
+      </c>
+      <c r="E12" s="1">
+        <v>-99.8</v>
+      </c>
+      <c r="F12" s="4">
+        <v>-0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" t="s">
+        <v>17</v>
+      </c>
+      <c r="B13" s="1">
+        <v>-125</v>
+      </c>
+      <c r="C13" s="2">
+        <v>0</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>-125.1</v>
+      </c>
+      <c r="F13" s="4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" t="s">
+        <v>18</v>
+      </c>
+      <c r="B14" s="1">
+        <v>-166</v>
+      </c>
+      <c r="C14" s="2">
+        <v>0</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>-166</v>
+      </c>
+      <c r="F14" s="4">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>